<commit_message>
docs: HANDOFF.md 충돌 해결 + start-admin.ps1 환경변수 추가
- HANDOFF.md: rebase 충돌 해결 (upstream platform 세션 노트 보존)
- start-admin.ps1: ONPREM_BASE_URL / AWS_DEFAULT_REGION / LIFESYNC_RAW_S3_BUCKET 환경변수 추가
- project-progress.md: VPN 재구성 주의사항 + admin 배포 경로 확정 내용 갱신

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/관리자_대시보드_설계서_V5_3.xlsx
+++ b/관리자_대시보드_설계서_V5_3.xlsx
@@ -495,7 +495,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" style="7" min="1" max="1"/>
     <col width="36" customWidth="1" style="7" min="2" max="2"/>
@@ -760,7 +760,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>SUM(purchased_flag='Y') / COUNT(*) * 100 — 전체 누적 노출(추천) 대비 구매 전환율 (클릭 기반 아님)</t>
+          <t>SUM(purchased_flag='Y') / SUM(clicked_flag='Y') * 100</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
     <row r="17" ht="37.2" customHeight="1" s="7">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>온프레미스</t>
+          <t>On-Premises</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1375,7 +1375,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4" outlineLevelCol="0"/>
   <cols>
     <col width="37.59765625" customWidth="1" style="7" min="1" max="1"/>
     <col width="36" customWidth="1" style="7" min="2" max="2"/>
@@ -2236,8 +2236,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" style="7" min="1" max="1"/>
     <col width="36" customWidth="1" style="7" min="2" max="2"/>
@@ -2285,12 +2285,12 @@
     <row r="3" ht="43.2" customHeight="1" s="7">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>추천 CTR (클릭률)</t>
+          <t>추천 CTR</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>노출 대비 클릭률 — 추천 효율 KPI (최근 1일)</t>
+          <t>노출 대비 클릭률 — 추천 효율 KPI</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2300,24 +2300,24 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>customer_recommend_daily</t>
+          <t>customer_recommend_history</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>SUM(clicked_flag='Y') / COUNT(*) * 100 — 최근 1일</t>
+          <t>SUM(clicked_flag='Y') / COUNT(*) * 100 — 최근 N일</t>
         </is>
       </c>
     </row>
     <row r="4" ht="58.2" customHeight="1" s="7">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>거래율 CVR (전환)</t>
+          <t>구매 전환율 CVR</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>노출 대비 구매 전환율 (최근 1일)</t>
+          <t>클릭 대비 구매 전환율</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2327,29 +2327,29 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>customer_recommend_daily</t>
+          <t>customer_recommend_history</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>SUM(purchased_flag='Y') / COUNT(*) * 100 — 최근 1일. 노출(추천 수) 대비 CVR</t>
+          <t>SUM(purchased_flag IN ('Y','1')) * 100.0 / COUNT(*) — 주의: 추천 수(노출) 대비 CVR. 클릭 수 대비 아님</t>
         </is>
       </c>
     </row>
     <row r="5" ht="59.4" customHeight="1" s="7">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>마지막 배치 갱신</t>
+          <t>AI 평균 예측 확신도</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Vertex AI → DDB 마지막 배치 갱신 완료 시각</t>
+          <t>AI 평균 예측 확신도 (vip / signup / rec)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>AWS DynamoDB</t>
+          <t>AWS DynamoDB scan</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Scan Limit=1 · ProjectionExpression=update_time — 가장 최근 update_time 반환</t>
+          <t>AVG(vip_prob, signup_prob, rec_prob) — 3 확률 평균</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>DynamoDB 전체 레코드 수 = Vertex AI 배치 처리 완료 고객 수</t>
+          <t>동의 완료 + 가입 완료 교집합 (AI 학습 대상)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Scan COUNT(Items) — 조건 필터 없음. 배치 갱신 완료 고객 수 그대로</t>
+          <t>Scan COUNT(Items) — 동의/가입 조건 DDB 필터 없음. 정확한 분석 대상 수는 On-Prem 별도 집계 필요</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>일별 CTR=SUM(clicked_flag='Y')/COUNT(*) · CVR=SUM(purchased_flag='Y')/COUNT(*) ×100 — GROUP BY DATE(recommended_at)</t>
+          <t>일별 CTR=SUM(clicked_flag='Y')/COUNT(*) · CVR=SUM(purchased_flag='Y')/NULLIF(SUM(clicked_flag='Y'),0) ×100 — GROUP BY DATE(recommended_at)</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>customer_recommend_history JOIN product_master JOIN category_master cat</t>
+          <t>category_master</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>GROUP BY cat.category_code ORDER BY recommended DESC LIMIT 10 — 최근 7일. _aurora_category_ctr_donut()</t>
+          <t>GROUP BY category_code</t>
         </is>
       </c>
     </row>
@@ -2613,17 +2613,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>On-Prem /internal/profile/list-all 직접 HTTP (1순위) / AWS DynamoDB analytics_segment_performance (fallback)</t>
+          <t>On-Prem Lambda (1순위) / AWS DynamoDB analytics_segment_performance (fallback)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>On-Prem GET /internal/profile/list-all?size=500&amp;after=&lt;cursor&gt; → Aurora customer_recommend_history WHERE global_id IN(age_band list)</t>
+          <t>list_by_age_band action → Aurora customer_recommend_history WHERE global_id IN(age_band 샘플)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2-step: OnPrem /internal/profile/list-all 직접 페이지네이션 (cursor: next_after, size=500, max 10 pages, timeout=2s/call) → age_groups dict 빌드 → Aurora GROUP BY global_id IN() ; OnPrem 실패 시 analytics_segment_performance age_band# prefix fallback. _ai_age_perf_2step() V6 R21</t>
+          <t>2-step: OnPrem list_by_age_band → Aurora GROUP BY global_id IN() ; OnPrem 실패 시 analytics_segment_performance age_band# prefix fallback. _ai_age_perf_2step()</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
     <row r="23" ht="25.95" customHeight="1" s="7">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>빅쿼리 분석 (5번 영역, 3 카드)</t>
+          <t>BigQuery 분석 (5번 영역, 3 카드)</t>
         </is>
       </c>
     </row>
@@ -2830,15 +2830,15 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="43.2" customHeight="1" s="7">
+    <row r="32" ht="65.40000000000001" customHeight="1" s="7">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>정밀도 (Precision)</t>
+          <t>Precision / Recall</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>추천 중 실제 클릭된 비율 — 70% 기준 색상 표시 (green/red). Recall 제거: 폐쇄형 추천 UI에서 사용자가 추천 상품만 보므로 FN=0 고정 → Recall 항상 100%, 지표 무의미</t>
+          <t>VIP / Churn / NBA 모델 평가</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>model_name / precision_score — ORDER BY eval_date DESC LIMIT 4. _aurora_pr_models(). recall_score 컬럼 쿼리 제거됨</t>
+          <t>model_name / precision_score / recall_score — ORDER BY eval_date DESC LIMIT 4. _aurora_pr_models()</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2909,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>상단 4 KPI (CTR · CVR · 마지막 배치 갱신 · 분석 대상 고객)</t>
+          <t>상단 4 KPI</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Aurora customer_recommend_daily (CTR/CVR 최신 1일) + DDB Limit=1 (마지막 배치 갱신 update_time) + DDB Scan COUNT (분석 대상 고객 수). _ai_kpi4_from_aws()</t>
+          <t>Aurora customer_recommend_history GROUP BY DATE = CURDATE() (CTR/CVR 당일 실시간 집계) + DDB Scan (분석 대상 count). _ai_kpi4_from_aws() — customer_recommend_daily 미사용</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3157,154 +3157,6 @@
       <c r="G42" s="3" t="inlineStr">
         <is>
           <t>인구통계 카드 영역 — 도넛/표 부분 갱신</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>GET /api/ai/chart/trend</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>7일 추천 성과 추이 SVG fragment (server-rendered)</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>admin-platform/app.py · api_ai_chart_trend()</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>/api/ai/chart/trend</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Aurora customer_recommend_history GROUP BY DATE(recommended_at) 최근 7일 — 실패 시 빈 차트. _aurora_recommend_trend_7day()</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>JS 폴링 30s</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>&lt;div id="ai-chart-trend"&gt; innerHTML 교체 (server-rendered SVG)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>GET /api/ai/chart/donut</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>카테고리별 도넛 CTR SVG fragment (server-rendered)</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>admin-platform/app.py · api_ai_chart_donut()</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>/api/ai/chart/donut</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Aurora customer_recommend_history JOIN product_master JOIN category_master GROUP BY category_code LIMIT 10 — 최근 7일. _aurora_category_ctr_donut()</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>JS 폴링 30s</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>&lt;div id="ai-chart-donut"&gt; innerHTML 교체</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>GET /api/ai/chart/age</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>연령대별 추천 성과 진행바 SVG fragment (server-rendered)</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>admin-platform/app.py · api_ai_chart_age()</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>/api/ai/chart/age</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>On-Prem /internal/profile/list-all 페이지네이션 → Aurora customer_recommend_history WHERE global_id IN() / DDB analytics_segment_performance fallback. _ai_age_perf_2step() V6 R21</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>JS 폴링 30s</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>&lt;div id="ai-chart-age"&gt; innerHTML 교체</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>GET /api/ai/chart/histogram</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>AI 예측 분포 히스토그램 SVG fragment (server-rendered)</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>admin-platform/app.py · api_ai_chart_histogram()</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>/api/ai/chart/histogram</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>DDB lifesync_customer_result scan(ProjectionExpression=dynamic_score) — 5 bucket: 0-20/20-40/40-60/60-80/80-100</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>JS 폴링 30s</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>&lt;div id="ai-chart-histogram"&gt; innerHTML 교체</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3181,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J39"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" style="7" min="1" max="1"/>
     <col width="36" customWidth="1" style="7" min="2" max="2"/>
@@ -3343,7 +3195,7 @@
     <row r="1" ht="25.95" customHeight="1" s="7">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>AWS 5 VPC (1번 영역, 5 카드)</t>
+          <t>AWS 3 VPC (1번 영역, 3 카드)</t>
         </is>
       </c>
     </row>
@@ -3455,274 +3307,272 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AWS 웨어러블 VPC</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kinesis Stream · Wearable EC2</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>AWS describe APIs</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>vpc-* + Kinesis + Wearable EC2</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>실시간 웨어러블 데이터 수신 VPC. VPC Name tag lifesync-wearable-vpc 기반 자동 발견. deploy_group=wearable 분류</t>
-        </is>
-      </c>
-    </row>
     <row r="7" ht="25.95" customHeight="1" s="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AWS 관리 VPC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Admin EC2 (Windows Server 2022) — 관리자 대시보드 플랫폼</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>AWS describe APIs</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>vpc-* + Admin EC2</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>관리자 플랫폼 EC2 전용 VPC (10.4.0.0/16 · admin subnet 10.4.20.0/24). VPC Name tag lifesync-management-vpc 기반. deploy_group=management 분류</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1" s="7"/>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Connectivity / GCP / On-Prem (2번 영역, 3 카드)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" s="7">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>기능</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>데이터 소스</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>테이블 / 객체</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>컬럼 / 비고</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="37.2" customHeight="1" s="7">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>연결 현황 · GCP · 온프레미스 (2번 영역, 3 카드)</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>AWS Connectivity</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>TGW · VPN · VPC Peering</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>AWS EC2 describe</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>tgw-* / vpn-* / vpc-peering</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>tgw / vpn / vpc-peering 상태</t>
         </is>
       </c>
     </row>
     <row r="10" ht="41.4" customHeight="1" s="7">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>기능</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>설명</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>데이터 소스</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>테이블 / 객체</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>컬럼 / 비고</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>GCP</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>BigQuery · Vertex AI · Cloud Run</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>GCP Cloud Monitoring</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BigQuery + Vertex AI + Cloud Run</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>GCP 자격증명으로 헬스 체크</t>
         </is>
       </c>
     </row>
     <row r="11" ht="35.4" customHeight="1" s="7">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AWS 연결 현황</t>
+          <t>On-Prem</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>TGW · VPN (VPC Peering 제거됨)</t>
+          <t>ls-db · ls-token · ls-api 헬스</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>AWS EC2 describe</t>
+          <t>PrivateAPI (VPN 경유)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>tgw-* / vpn-*</t>
+          <t>ls-db / ls-token / ls-api</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>TGW / VPN 상태. VPC Peering API 코드 삭제됨</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="38.4" customHeight="1" s="7">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>GCP</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>BigQuery · Vertex AI · Cloud Run</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>GCP Cloud Monitoring</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BigQuery + Vertex AI + Cloud Run</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>GCP 자격증명으로 헬스 체크</t>
+          <t>strongSwan VPN 통한 ping</t>
         </is>
       </c>
     </row>
     <row r="13" ht="25.95" customHeight="1" s="7">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>온프레미스</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ls-db · ls-token · ls-api 헬스</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>PrivateAPI (VPN 경유)</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ls-db / ls-token / ls-api</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>strongSwan VPN 통한 ping</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1" s="7"/>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Wearable 실시간 (3번 영역, KPI 4 + 표 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" s="7">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>기능</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>데이터 소스</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>테이블 / 객체</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>컬럼 / 비고</t>
+        </is>
+      </c>
+    </row>
     <row r="15" ht="39" customHeight="1" s="7">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>웨어러블 실시간 (3번 영역, KPI 4 + 표 2)</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>활성 디바이스</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>최근 1초 송신 디바이스 수</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>AWS Kinesis Stream + DynamoDB</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>wearable_latest{global_id}</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Kinesis consumer 가 매 batch 100 record DDB 갱신</t>
         </is>
       </c>
     </row>
     <row r="16" ht="40.8" customHeight="1" s="7">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>기능</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>설명</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>데이터 소스</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>테이블 / 객체</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>컬럼 / 비고</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>송신율</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>활성 / 등록 %</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>AWS Kinesis Stream</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>IncomingRecords (5분 윈도우)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>IncomingRecords / 등록 디바이스 수 × 100</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1" s="7">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>활성 디바이스</t>
+          <t>건강 RED 카운트</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>최근 1초 송신 디바이스 수</t>
+          <t>AHA/WHO 임상 임계 위반 (즉시 조치)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>AWS Kinesis Stream + DynamoDB</t>
+          <t>AWS DynamoDB anomaly_event</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>wearable_latest{global_id}</t>
+          <t>anomaly_event scan (today)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Kinesis consumer 가 매 batch 100 record DDB 갱신</t>
+          <t>HR&lt;50 / HR≥120 / SpO2&lt;90 / stress≥76</t>
         </is>
       </c>
     </row>
     <row r="18" ht="39" customHeight="1" s="7">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>송신율</t>
+          <t>건강 YELLOW 카운트</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>활성 / 등록 %</t>
+          <t>경계 영역 (모니터링)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>AWS Kinesis Stream</t>
+          <t>AWS DynamoDB anomaly_event</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>IncomingRecords (5분 윈도우)</t>
+          <t>anomaly_event scan (today)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>IncomingRecords / 등록 디바이스 수 × 100</t>
+          <t>HR 50-59 또는 101-119 / SpO2 90-94 / stress 51-75</t>
         </is>
       </c>
     </row>
     <row r="19" ht="37.2" customHeight="1" s="7">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>건강 위험 카운트</t>
+          <t>🔴 건강 RED 표</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>AHA/WHO 임상 임계 위반 (즉시 조치)</t>
+          <t>최근 10건 — 시각/gid/이름/심박/SpO2/스트레스/사유 컬럼</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3732,24 +3582,24 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>anomaly_event scan (today)</t>
+          <t>anomaly_event (PK: global_id, SK: event_time)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>HR&lt;50 / HR≥120 / SpO2&lt;90 / stress≥76</t>
+          <t>시계열 알람 로그 — 시간순 정렬, 화면 상위 10개</t>
         </is>
       </c>
     </row>
     <row r="20" ht="37.8" customHeight="1" s="7">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>건강 주의 카운트</t>
+          <t>🟡 건강 YELLOW 표</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>경계 영역 (모니터링)</t>
+          <t>경계 영역 최근 10건 — RED 표와 동일 컬럼 구조 (severity=YELLOW)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3759,250 +3609,218 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>anomaly_event scan (today)</t>
+          <t>anomaly_event filter by severity</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>HR 50-59 또는 101-119 / SpO2 90-94 / stress 51-75</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="38.4" customHeight="1" s="7">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>🔴 건강 위험 표</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>최근 10건 — 시각/gid/이름/심박/SpO2/스트레스/사유 컬럼</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>AWS DynamoDB anomaly_event</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>anomaly_event (PK: global_id, SK: event_time)</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>시계열 알람 로그 — 시간순 정렬, 화면 상위 10개</t>
+          <t>동일 (severity=YELLOW)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="25.95" customHeight="1" s="7">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>🟡 건강 주의 표</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>경계 영역 최근 10건 — RED 표와 동일 컬럼 구조 (severity=YELLOW)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>AWS DynamoDB anomaly_event</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>anomaly_event filter by severity</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>동일 (severity=YELLOW)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1" s="7"/>
-    <row r="24" ht="42.6" customHeight="1" s="7"/>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Network API 엔드포인트 (4번 영역, 하단 list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="7">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>기능</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>데이터 소스</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>테이블 / 객체</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>컬럼 / 비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42.6" customHeight="1" s="7">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Network 라우트 표</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>TGW / VPN / VM / Kinesis / EMR / Local Lab</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>admin 라우트 메타</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Network API 9 엔드포인트</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>9 라우트 listing — name / method / desc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="25.95" customHeight="1" s="7">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>🌐 API — 화면 데이터 호출 (V5 신설: 호출 주기 + 표시 방식)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="25.95" customHeight="1" s="7">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="27" ht="24" customHeight="1" s="7">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>API</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>구현 위치</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>엔드포인트</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>데이터 소스</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>호출 주기</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>표시 방식</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1" s="7">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>GET /stream/wearable</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Wearable 실시간 — KPI 4 + RED/YELLOW 표</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>admin-platform/app.py · stream_wearable()</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>/stream/wearable</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>wearable_engine.snapshot() — mock_wearable_batch.json 적재 + 1초 tick 메모리 시뮬레이션 (운영 전환 시: Kinesis consumer로 교체 예정)</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>SSE 1s push</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>&lt;tbody&gt; innerHTML 교체 + KPI textContent + ts-we-* 3건</t>
         </is>
       </c>
     </row>
     <row r="28" ht="91.2" customHeight="1" s="7">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GET /api/ops/wearable</t>
+          <t>GET /stream/wearable</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>SSE 폴백 (단발 JSON)</t>
+          <t>Wearable 실시간 — KPI 4 + RED/YELLOW 표</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>admin-platform/app.py · api_ops_wearable()</t>
+          <t>admin-platform/app.py · stream_wearable()</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>/api/ops/wearable</t>
+          <t>/stream/wearable</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>wearable_engine.snapshot() — 동일 메모리 엔진 (SSE 비대응 클라이언트용 단발 JSON 폴백)</t>
+          <t>wearable_engine.snapshot() — mock_wearable_batch.json 적재 + 1초 tick 메모리 시뮬레이션 (운영 전환 시: Kinesis consumer로 교체 예정)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>수동 호출</t>
+          <t>SSE 1s push</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>SSE 비대응 클라이언트용 — 화면 자동 호출 X</t>
+          <t>&lt;tbody&gt; innerHTML 교체 + KPI textContent + ts-we-* 3건</t>
         </is>
       </c>
     </row>
     <row r="29" ht="58.2" customHeight="1" s="7">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GET /api/network/tgw</t>
+          <t>GET /api/ops/wearable</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Transit Gateway 상태</t>
+          <t>SSE 폴백 (단발 JSON)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>admin-platform/app.py · api_network_tgw</t>
+          <t>admin-platform/app.py · api_ops_wearable()</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>/api/network/tgw</t>
+          <t>/api/ops/wearable</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>EC2 describe_transit_gateways + attachments</t>
+          <t>wearable_engine.snapshot() — 동일 메모리 엔진 (SSE 비대응 클라이언트용 단발 JSON 폴백)</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>JS 폴링 30s</t>
+          <t>수동 호출</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>TGW 헬스 카드 (R13 Connectivity)</t>
+          <t>SSE 비대응 클라이언트용 — 화면 자동 호출 X</t>
         </is>
       </c>
     </row>
     <row r="30" ht="49.8" customHeight="1" s="7">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GET /api/network/vpn</t>
+          <t>GET /api/network/tgw</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>VPN 터널 상태</t>
+          <t>Transit Gateway 상태</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>admin-platform/app.py · api_network_vpn</t>
+          <t>admin-platform/app.py · api_network_tgw</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>/api/network/vpn</t>
+          <t>/api/network/tgw</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>EC2 describe_vpn_connections + VgwTelemetry</t>
+          <t>EC2 describe_transit_gateways + attachments</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -4012,34 +3830,34 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>VPN 헬스 카드 (R13 Connectivity)</t>
+          <t>TGW 헬스 카드 (R13 Connectivity)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="43.8" customHeight="1" s="7">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GET /api/vm/group</t>
+          <t>GET /api/network/vpn</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Group VM EC2 (6 계열사)</t>
+          <t>VPN 터널 상태</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>admin-platform/app.py · api_vm_group</t>
+          <t>admin-platform/app.py · api_network_vpn</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>/api/vm/group</t>
+          <t>/api/network/vpn</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>EC2 describe_vpcs(Name=lifesync-*-vpc) → VPC내 EC2 → deploy_group=group-app 필터. VPC Name에 group 포함 여부 분류</t>
+          <t>EC2 describe_vpn_connections + VgwTelemetry</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -4049,34 +3867,34 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>GroupVM VPC 카드 rows 갱신 (R9)</t>
+          <t>VPN 헬스 카드 (R13 Connectivity)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="81.59999999999999" customHeight="1" s="7">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GET /api/vm/wearable</t>
+          <t>GET /api/vm/group</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Wearable VM + Custom metric</t>
+          <t>Group VM EC2 (6 계열사)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>admin-platform/app.py · api_vm_wearable</t>
+          <t>admin-platform/app.py · api_vm_group</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>/api/vm/wearable</t>
+          <t>/api/vm/group</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>EC2 describe + CloudWatch LifeSync/Wearable namespace</t>
+          <t>EC2 describe_vpcs(Name=lifesync-*-vpc) → VPC내 EC2 → deploy_group=group-app 필터. VPC Name에 group 포함 여부 분류</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -4086,34 +3904,34 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Wearable VM 상태 (R20 송신율 sub 정보)</t>
+          <t>GroupVM VPC 카드 rows 갱신 (R9)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="43.8" customHeight="1" s="7">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GET /api/kinesis/status</t>
+          <t>GET /api/vm/wearable</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Kinesis 스트림 상태</t>
+          <t>Wearable VM + Custom metric</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>admin-platform/app.py · api_kinesis_status</t>
+          <t>admin-platform/app.py · api_vm_wearable</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>/api/kinesis/status</t>
+          <t>/api/vm/wearable</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Kinesis describe_stream</t>
+          <t>EC2 describe + CloudWatch LifeSync/Wearable namespace</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -4123,34 +3941,34 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Data VPC 카드 sub 정보 (R8)</t>
+          <t>Wearable VM 상태 (R20 송신율 sub 정보)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="46.2" customHeight="1" s="7">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GET /api/emr/status</t>
+          <t>GET /api/kinesis/status</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>EMR 클러스터 상태</t>
+          <t>Kinesis 스트림 상태</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>admin-platform/app.py · api_emr_status</t>
+          <t>admin-platform/app.py · api_kinesis_status</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>/api/emr/status</t>
+          <t>/api/kinesis/status</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>EMR list_clusters</t>
+          <t>Kinesis describe_stream</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -4160,204 +3978,205 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Data VPC 카드 sub 정보 (R8) — 현재 EMR 미배포</t>
+          <t>Data VPC 카드 sub 정보 (R8)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="39" customHeight="1" s="7">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>GET /api/emr/status</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>EMR 클러스터 상태</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>admin-platform/app.py · api_emr_status</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>/api/emr/status</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>EMR list_clusters</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>JS 폴링 30s</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Data VPC 카드 sub 정보 (R8) — 현재 EMR 미배포</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="67.8" customHeight="1" s="7">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>GET /api/admin/local-lab-status</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>On-Prem Local Lab 헬스</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>admin-platform/app.py · api_admin_local_lab_status</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>/api/admin/local-lab-status</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>PrivateAPI onprem-query local_lab_status action · `/api/local/status` 와 alias</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>JS 폴링 30s</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>On-Prem 카드 (R15) rows 갱신</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="67.8" customHeight="1" s="7">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="37" ht="60.6" customHeight="1" s="7">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>GET /api/cloud/status</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>AWS + GCP 통합 헬스 단건 (cloud3 와 별도 raw)</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>admin-platform/app.py · api_cloud_status</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>/api/cloud/status</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>AWS describe (6 서비스) + _stub_gcp_status (BigQuery/Vertex/Cloud Run)</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>JS 폴링 30s</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>Cloud Status 통합 헬스 — Connectivity 영역 (R11~R15)</t>
         </is>
       </c>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
-    </row>
-    <row r="37" ht="60.6" customHeight="1" s="7">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+    </row>
+    <row r="38" ht="19.8" customFormat="1" customHeight="1" s="5">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>GET /api/datavpc/status</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>DataVPC 4 컴포넌트 통합 상태 (신규)</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>admin-platform/app.py · api_datavpc_status()</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>/api/datavpc/status</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>S3 head_bucket + Kinesis describe_stream + Glue get_job_runs + EMR list_clusters — {s3_bucket, s3_state, kinesis, glue, emr}</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>JS 폴링 30s</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>Data VPC 카드 rows 갱신 (R8)</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="19.8" customFormat="1" customHeight="1" s="5">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="39" ht="76.8" customFormat="1" customHeight="1" s="3">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>GET /api/vm/platform</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Platform VPC EC2 인스턴스 (신규)</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>admin-platform/app.py · api_vm_platform()</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>/api/vm/platform</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>EC2 describe_vpcs(Name=lifesync-*-vpc) → VPC내 EC2 → deploy_group='platform' 필터 (vpc_name에 group/wearable 미포함)</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>JS 폴링 30s</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Platform VPC 카드 rows 갱신 (R7)</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="76.8" customFormat="1" customHeight="1" s="3">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>GET /api/vm/management</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>관리 VPC Admin EC2 인스턴스 상태</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>admin-platform/app.py · api_vm_management</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>/api/vm/management</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>EC2 describe_vpcs(Name=lifesync-*-vpc) → VPC내 EC2 → deploy_group='management' 필터 (vpc_name에 'management' 포함 여부)</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>JS 폴링 30s</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>관리 VPC 카드 rows 갱신</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A15:E15"/>
+  <mergeCells count="5">
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>